<commit_message>
feat(ref): 模板清单 template_matrix.tsv + 教程第11页签；修 utf8_stdio 重复包裹导致 stdout 被关
- reference/template_matrix.tsv: 10 份空白模板 × browse node 数 × 覆盖类目（预筛/全量）
- make_tutorial: 新增 11-模板清单 页签
- flatfile.utf8_stdio: 幂等，避免二次包裹后旧 wrapper 回收把 buffer 关掉（import pick_template 时踩到）
- pick_template: 只在 __main__ 时切 stdout，避免被 import 时副作用
</commit_message>
<xml_diff>
--- a/docs/教程.xlsx
+++ b/docs/教程.xlsx
@@ -18,6 +18,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08-文案样例" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09-枚举速查" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10-站点专属取值" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11-模板清单" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00-速查'!$A$1:$B$16</definedName>
@@ -31,6 +32,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08-文案样例'!$A$1:$E$121</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09-枚举速查'!$A$1:$G$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10-站点专属取值'!$A$1:$D$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'11-模板清单'!$A$1:$F$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3053,6 +3055,381 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>国家</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>模板文件</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>browse node 数</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>性质</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>覆盖类目</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>有数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>德国空白上传模版.xlsx</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>106</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>全量</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>bikini/monokini/tankini</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>惠全优 德国 2399.xlsm</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>预筛(单类目)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>bikini</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>比利时</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>比利时空白上传表.xlsm</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>全量</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>bikini/monokini/onepiece/tankini</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>法国空白上传模版.xlsm</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>113</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>全量</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>bikini/monokini/onepiece/tankini</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>1391.xlsm</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>全量</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>bikini/monokini/onepiece/tankini</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>英国空白上传模版.xlsm</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>全量</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>bikini/monokini/onepiece/tankini</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>takini set 模板.xlsm</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>预筛(单类目)</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>tankini</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>荷兰 monokini空白模版.xlsm</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>142</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>全量</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>bikini/monokini/onepiece/tankini</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>荷兰空白上传模版.xlsm</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>预筛(单类目)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>bikini</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>西班牙空白上传模版.xlsm</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>97</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>全量</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>bikini/monokini/onepiece/tankini</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>